<commit_message>
Add full platform answer text column to tracking xlsx
New column "Финальный ответ платформы (полный текст)" carries the
complete verbatim answer for each of the 25 rows (18 questions +
7 collection rechecks), as transcribed from each screenshot, rather
than the condensed "Ответ (кратко)" summary already present.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/accounts/eco/pilot-test-03-eco2-tracking.xlsx
+++ b/docs/accounts/eco/pilot-test-03-eco2-tracking.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -541,6 +541,7 @@
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="70" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -604,6 +605,11 @@
           <t>Статус (12.09.2026)</t>
         </is>
       </c>
+      <c r="M1" s="8" t="inlineStr">
+        <is>
+          <t>Финальный ответ платформы (полный текст)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -662,6 +668,16 @@
           <t>Без изменений — верно</t>
         </is>
       </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Как начальник склада вы должны:
+1. Организовать маркировку несоответствующих ТМЦ актом забраковки ТМЦ — форма 03-01. Упакованную паллету можно промаркировать четырьмя актами, разместив их с каждой стороны паллеты.
+2. Переместить ТМЦ в зону «БРАК» не позднее одного рабочего дня с момента получения акта.
+3. Разместить забракованные ТМЦ в соответствии с требованиями, указанными в акте забраковки. Продукцию, содержащую аллерген, размещают в зоне «БРАК_Аллерген».
+4. Перемещение ТМЦ на склад «БРАК» в базе 1С-8 организует бухгалтер по учёту ТМЦ.
+Источник: ПР-03-00-12 «Несоответствующая продукция», п. 5.7.4–5.7.5.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -720,6 +736,13 @@
           <t>Исправлено (vs 11.09)</t>
         </is>
       </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Процессом экспериментальной выработки управляет Технолог лаборатории: он руководит производственным процессом и при необходимости вносит корректировки в процесс производства, отражая их в РИ (форма 16-03).
+При отклонении показателей качества от нормируемых продукт дорабатывается под руководством Технолога лаборатории.
+Источник: И-16-01-11 «Внедрение новых видов продукции в производство», фрагмент с обязанностями Технолога лаборатории: «руководит производственным процессом на экспериментальной выработке».</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -778,6 +801,12 @@
           <t>Регрессия vs 12.09</t>
         </is>
       </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>В доступных источниках не нашёл инструкции, которая описывает действия мастера производства именно при пометке «Экспериментальная» в заказе. Найденный фрагмент касается проверки изменений заказа в 1С и не содержит порядка действий для экспериментальной партии.
+Источник найденного фрагмента: И-12-10-03 «Корректировка Заказу покупателя в 1С».</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -836,6 +865,16 @@
           <t>Исправлено на ЭКО_2</t>
         </is>
       </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Процессом экспериментальной выработки управляет Технолог лаборатории: он руководит производственным процессом и при необходимости вносит корректировки в процесс производства, отражая их в РИ (форма 16-03).
+Также:
+— Ведущий технолог ПО фиксирует в РИ отличия действий оператора и/или количества загруженных ингредиентов.
+— После выработки образец передаётся в ОКК для проверки качества.
+— При отклонении показателей качества продукт дорабатывается под руководством Технолога лаборатории.
+Источник: И-16-01/11, цитата: «Технолог лаборатории — руководит производственным процессом на экспериментальной выработке».</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -894,6 +933,16 @@
           <t>Без изменений — верно + аномалия</t>
         </is>
       </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>После завершения фасовки оператор ПО заполняет в «Рабочей инструкции на производство» (форма 16-03):
+— «Кол-во тарных мест» — фактическое количество расфасованного продукта в штуках для каждого вида характеристики номенклатуры;
+— «Общее количество» — фактически расфасованное количество готового продукта в килограммах;
+— «Дата» — дата окончания фасовки;
+— «Фасовщик ФИО подпись» — ФИО и подпись сотрудника, который фасовал продукт.
+Источник: И-08-02-10 «Фасовка и упаковка готовой продукции», раздел «Заполнение "Рабочей инструкции на производство"».</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -952,6 +1001,16 @@
           <t>Без изменений — ошибка сохраняется</t>
         </is>
       </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>При выпуске продукции с меньшим весом:
+1. Откройте Заказ.
+2. Создайте корректировку к Заказу.
+3. В корректировке укажите количество, которое нужно убрать из Заказа, со знаком «−».
+4. Поскольку по заказу имеется Заказ на производство, для изменения продукта следует обратиться к ОБ.
+Источник: документ «И-12-10-03 Корректировка Заказу покупателя в 1С», таблица «Описание процесса оформления Заказа и Действий в Корректировке к Заказу в 1С». В найденном фрагменте отдельно не указано, как рассчитывать величину уменьшения именно в килограммах.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1010,6 +1069,20 @@
           <t>Исправлено на ЭКО_2</t>
         </is>
       </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>При сдаче заказа на производство с уменьшением веса:
+1. В «Заказе на производство» нажмите «Ввести на основании» → «Корректировка заказа на производство».
+2. На вкладке «Продукция и услуги»: в первой строке уменьшите количество готовой продукции на вес, равный тарному месту; во второй строке добавьте вес вскрытого тарного места без прикрепления к заказу покупателя.
+3. На вкладке «Материалы» удалите все строки.
+4. Проведите корректировку.
+5. В «Заказе на производство» нажмите «Анализ» и сверяйте получившийся вес с весом в форме 16-03 «Рабочая инструкция на производство».
+6. Далее заполните вкладку «Дополнительно»: укажите исполнителя, фактически использованное оборудование и дату исполнения заказа.
+7. Во вкладке «Процесс» установите отметку «Фасовка»; если не нажата кнопка «Выгрузка WMS», нажмите её.
+8. Заполните в форме 08-03 «Карточка выпуска готовой продукции» поле «раздел передачи готовой продукции с производства на склад».
+Источник: Д-08-04/01 «Проведение корректировок к заказу на производство в базе 1С-8 при сдаче готовой продукции на склад», пп. 3.4–3.5.6.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1068,6 +1141,12 @@
           <t>Исправлено + аномалия</t>
         </is>
       </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Для пластиковой тары объёмом свыше 1,5 до 5 л включительно высота падения должна быть не менее 0,8 м.
+Источник: Методика №38, «Высота падения, м, не менее: для значения свыше 1,5 до 5 включительно — 0,8».</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1126,6 +1205,12 @@
           <t>Аномалия воспроизведена при верном скоупе</t>
         </is>
       </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Для пластиковой тары объёмом свыше 1,5 до 5 литров включительно высота падения должна быть не менее 0,8 м.
+Источник: Методика №38, файл для теста ИИ (1)/Методика №38.doc: «Высота падения, м, не менее: для значения свыше 1,5 до 5 включительно — 0,8». (Повтор при явно подтверждённом скоупе: только Документы, SQL/каталог выключен, коллекция ЭКО.)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1184,6 +1269,17 @@
           <t>Без изменений — верно</t>
         </is>
       </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Технолог ПО получает сырьё так:
+1. Согласовывает с мастером ПО приоритетность задач на день.
+2. В 1С8 во вкладке «Процесс» соответствующего заказа устанавливает флажок «Передать сырьё» и нажимает «Выгрузить WMS».
+3. Дублирует запрос по телефону сотруднику СО, называя номера заказов и время, к которому нужно передать сырьё.
+4. После обратной связи от сотрудника СО о перемещении сырья забирает его на участке выдачи и перемещает к соответствующему оборудованию.
+Сырьё выдаётся на основании «Карточки выпуска готовой продукции» (форма 08-03), подписанной кладовщиком СО. При отсутствии в 1С8 отметки «Подбор сырья завершён» технолог ПО должен немедленно связаться по телефону с сотрудником СО, сообщить номер заказа о срочной сборке и передаче сырья, а затем проинформировать ответственного сотрудника ПО.
+Источник: Д-08-07/01 «Порядок получения ТМЦ с "Участка выдачи сырья" и сдача ТМЦ...», п. 5.1–5.4; ПР-08-00-14 «Производственный процесс», п. 5.4.4.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1242,6 +1338,17 @@
           <t>Частично улучшено (как на 12.09)</t>
         </is>
       </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Если заявка на комплектацию уже распечатана:
+1. Сообщите сотрудникам ОД и начальнику СО, что в заказ необходимо внести изменение.
+2. Откорректируйте заказ покупателя по И-12-10-03: откройте заказ и создайте корректировку; оставьте строку с исходной номенклатурой, которую нужно убрать; новой строкой добавьте ту же номенклатуру с требуемой характеристикой; при необходимости заполните материалы по спецификации и проведите корректировку.
+3. После внесения изменений уведомьте сотрудников ОД и начальника СО по электронной почте или телефону.
+4. Сотрудники ОД распечатают обновлённую заявку на комплектацию, передадут её в СО и повторно установят отметку «Заявка на комплектацию распечатана».
+Если по заказу уже создан заказ на производство, для изменения продукта нужно обратиться к ОБ.
+Источники: И-12-10-03 «Корректировка заказа покупателя в 1С»; И-12-12-06 «Оформление заказа покупателя».</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1300,6 +1407,16 @@
           <t>Улучшено на ЭКО_2 (не дословно как предсказано)</t>
         </is>
       </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Как начальник склада (СО), после получения акта забраковки вы должны:
+1. Организовать маркировку несоответствующих или потенциально небезопасных ТМЦ «Актом забраковки ТМЦ» (Форма 03-01). Упакованную паллету допускается маркировать четырьмя актами — по одному с каждой стороны.
+2. Переместить ТМЦ в складскую зону «БРАК» не позднее 1 рабочего дня с момента получения акта.
+3. Разместить забракованные ТМЦ в соответствии с требованиями, указанными в акте.
+Перемещение ТМЦ на склад «БРАК» в базе 1С-8 организует бухгалтер по учёту ТМЦ.
+Источник: инструкция 03-00-12, п. 5.7.4–5.7.5: «Начальник СО организует маркировку…» и «перемещение ТМЦ на складе в зону «БРАК», не позднее 1 рабочего дня…».</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1358,6 +1475,12 @@
           <t>Без изменений — верно</t>
         </is>
       </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Как начальник склада (СО), после получения акта забраковки вы должны: организовать маркировку несоответствующих ТМЦ (Форма 03-01), переместить их в зону «БРАК» не позднее 1 рабочего дня, разместить по требованиям акта.
+Источник: ПР-03-00-12, п. 5.7.4–5.7.5.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1416,6 +1539,17 @@
           <t>Без изменений — верное «не найдено»</t>
         </is>
       </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>При обнаружении забракованной продукции действуют так:
+1. Оператор ПО прекращает производство и сообщает Мастеру ПО и Технологу ПО. Если причина — попадание инородного предмета, выпуск также прекращается, а продукция считается потенциально небезопасной. Источник: И-08-03-09 «Действия при нештатных ситуациях».
+2. Мастер ПО: если продукция уже расфасована — организует её изоляцию; если продукция ещё не расфасована — сообщает Ведущему технологу ПО, Начальнику ПУ или Техническому директору. Источник: И-08-03-09, таблица №1.
+3. Решение о признании продукции несоответствующей принимает Руководитель ОКК / Директор по качеству. Результат фиксируется в соответствующем журнале, а также могут оформляться: Акт забраковки ТМЦ — форма 03-01; Акт разрешения на отклонение — форма 03-02; Акт на утилизацию — форма 03-04; запись в журнале «Учёт несоответствий продукции, сырья, тары» — форма 03-03. Источник: ПР-03-00-12 «Несоответствующая продукция».
+4. Ведущий технолог ПО действует согласно процедурам ПР-17-00 и ПР-03-00, а при необходимости сообщает группе БПП. Группа БПП действует согласно ПР-04-00. Источник: И-08-03-09, таблица №1.
+5. Решение о дальнейшем применении сырья и корректирующих действиях принимает Руководитель / Директор по качеству. Источник: ПР-03-00-12, таблица №1.
+Если акт уже передан на склад, начальник склада организует маркировку ТМЦ актом формы 03-01 и перемещение в зону «БРАК» не позднее одного рабочего дня; размещение выполняется по требованиям акта. Перемещение в 1С-8 организует бухгалтер по учёту ТМЦ. Источник: ПР-03-00-12, п. 5.7.4–5.7.5.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1474,6 +1608,12 @@
           <t>Консистентно на обеих коллекциях</t>
         </is>
       </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>В доступных источниках не нашёл указания на марку стретч-плёнки, которой обматывают паллеты с готовой продукцией.
+Источник найденного фрагмента — Д-09-01-17 «План контроля тары и упаковки», но в нём стретч-плёнка и её марка не указаны.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1532,6 +1672,12 @@
           <t>Без изменений — открытый вопрос</t>
         </is>
       </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>В доступных источниках не нашёл указания на марку стретч-плёнки для обмотки паллет с готовой продукцией.
+Источник проверенного документа — форма 09-01 «План контроля тары и упаковки», файл eco-converted-for-upload/forma-09-01-plan-kontrolya-tary-i-upakovki.docx: перечислены виды тары и упаковки, но стретч-плёнка и её марка не указаны.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1590,6 +1736,12 @@
           <t>Без изменений — верное «не найдено» + аномалия</t>
         </is>
       </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>В доступных источниках не нашёл указания, как часто нужно оценивать квалификацию внештатных сотрудников, работающих по договору подряда. Найденная процедура ПР-14-00-12 «Компетентность персонала» описывает оценку сотрудников, но найденные фрагменты не устанавливают периодичность для работников по договору подряда.
+Источник: ПР-14-00-12 «Компетентность персонала».</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1648,6 +1800,13 @@
           <t>Без изменений — верно + неполная карточка</t>
         </is>
       </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>В доступном фрагменте нет перечня полей журнала «Учёт уборки производственного оборудования» (форма 17-08).
+Найдено только, что форма 17-08 используется как чек-лист проверки ППУ и санитарного состояния производства, а еженедельный контроль состояния уборочного инвентаря проводит ответственный сотрудник ПО.
+Источник: И-08-04-13 «Уборка чистой зоны», фрагмент п. 4.4.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1706,6 +1865,16 @@
           <t>Без изменений — ошибка сохраняется (контрольный случай)</t>
         </is>
       </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Получить сырьё со склада «Проверка ОКК» можно после решения ОКК о его соответствии:
+1. Дождаться завершения контроля сырья сотрудником ОКК.
+2. После соответствия требованиям сотрудник ОКК по электронной почте информирует Руководителя ОКК, ответственных сотрудников бухгалтерии, Начальника СО и оператора склада с просьбой переместить сырьё со склада «На проверке ОКК» на соответствующий склад.
+3. После перемещения получить сырьё с обычного склада в установленном порядке.
+Решение о соответствии или несоответствии сырья принимает Руководитель ОКК / Директор по качеству. Самостоятельная выдача сырья технологу непосредственно со склада «Проверка ОКК» в источнике не предусмотрена.
+Источники: ПР-09-00-14 «Контроль качества»; ПР-03-00-12 «Несоответствующая продукция».</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1764,6 +1933,12 @@
           <t>ИСПРАВЛЕНО на ЭКО_2 (n=1/1 на тот момент)</t>
         </is>
       </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>В доступных источниках не нашёл порядка определения очередности выполнения нескольких срочных заявок на ремонт механиком.
+Источник найденного поиска — документы по корректировке заказов в 1С; они не описывают приоритизацию ремонтных заявок.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1822,6 +1997,13 @@
           <t>Без изменений — верно + аномалия</t>
         </is>
       </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Если поступило несколько заявок на обслуживание, первой выполняется заявка, неисправность по которой может повлиять на безопасность выпускаемой продукции.
+Приоритетность определяет Начальник ПУ и/или Мастер ПО. Заявки выполняет сотрудник РМС, назначенный Старшим механиком.
+Источник: ПР-10(02)-00/01 «Ремонтно-механическая служба»: «В случае наличия нескольких заявок на обслуживание приоритет отдается тем, которые способны оказать влияние на безопасность выпускаемой продукции. Приоритетность определяет Начальник ПУ и/или Мастер ПО».</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1880,6 +2062,17 @@
           <t>Без изменений — верно</t>
         </is>
       </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>При выпуске продукции с меньшим весом нужно сделать запас продукции на склад с учётом текущей загруженности оборудования:
+1. Проверьте отчёт «Планирование наработки на склад».
+2. Проверьте «Отчёт о загруженности оборудования» — он показывает статус оборудования по заказам и контрагентам.
+3. Учтите срочный заказ покупателя при составлении очередности производства; в найденном фрагменте отдельный порядок переприоритизации или остановки срочного заказа не установлен.
+4. Если потребность в запасе сформирована руководством, она передаётся Начальнику ПО запиской по электронной почте.
+5. Наработку на склад планируйте для товарных позиций с отметкой «не подлежит частичному резервированию».
+Источник: И-08-08-01 «Наработка складских позиций», файл для теста ИИ (1)/И-08-08-01 Наработка складских позиций.docx: «ПО планирует и осуществляет наработку складских позиций» на основании отчётов «планирование наработки на склад» и «Отчёт о загруженности оборудования»; потребность может быть передана Начальнику ПО руководством Компании.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1938,6 +2131,24 @@
           <t>Без изменений — ошибка сохраняется</t>
         </is>
       </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>Действия оператора ПО при фасовке готовой продукции:
+Перед фасовкой
+1. Проверить в «Рабочей инструкции на производство» (форма 16-03): поле «Примечания к тех. процессу» — дополнительные этикетки, специальные знаки и другая важная информация; поле «Вид фасовки» — характеристики номенклатуры, в которые нужно расфасовать продукцию.
+2. Осмотреть тару или упаковку: проверить её количество, качество, чистоту и целостность.
+3. Не выполнять фасовку на полу: минимальное расстояние от пола — 10 см.
+Источник: И-08-02-10 «Фасовка и упаковка готовой продукции», п. 3.1.1–3.1.2 и фрагмент раздела 3.3.
+В процессе и после фасовки
+4. После фасовки закрыть тару: канистру закрутить пробкой до характерного «щелчка» либо закрыть крышкой и простучать киянкой; при нарушении кольца, отсутствии полимерного вкладыша или перекосе пробки/крышки установить новую крышку.
+5. При фасовке порошковых форм упаковать пакет в соответствии с видом упаковки, указанным в форме 16-03: запаять пакеты размеров 20×35, 35×50, 40×80 и все металлизированные пакеты; пакет размера 80×110 затянуть хомутом.
+6. При обнаружении брака упаковки выполнить перефасовку. Если обнаружено несколько единиц бракованной упаковки — уведомить Мастера ПО/Технолога ПО/Начальника ПУ.
+7. После завершения фасовки заполнить в форме 16-03: «Кол-во тарных мест» — фактическое количество расфасованного продукта в штуках по каждому виду характеристики; «Общее количество» — фактическое количество готового продукта в килограммах; «Дата» — дату окончания фасовки; «Фасовщик ФИО подпись» — ФИО и подпись фасовавшего сотрудника.
+8. Вывезти этикированную готовую продукцию на паллете в зону передачи готовой продукции на склад.
+9. Передать ответственному сотруднику ПО полностью заполненную форму 16-03 с фактическим количеством расфасованной продукции.
+Источники: И-08-02-10, разделы 3-4; ПР-08-00-14 «Производственный процесс», п. 5.6.3 и 5.7.1.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1996,6 +2207,16 @@
           <t>ИСПРАВЛЕНО на ЭКО_2 (n=2/2)</t>
         </is>
       </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>Если утверждённой спецификации для нужной характеристики готовой продукции нет, ответственный сотрудник ПО должен:
+1. Направить запрос по электронной почте Ведущему технологу ПО.
+2. Поставить в копию Технического директора / Начальника ПО.
+3. Ведущий технолог ПО в течение одного рабочего дня вносит спецификацию для всех имеющихся характеристик номенклатуры.
+Подробный порядок самостоятельного добавления спецификации в интерфейсе 1С-8 в доступном фрагменте не приведён.
+Источник: Д-08-03-01 «Формирование заказов на производство в базе 1С-8», п. 3.6.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -2052,6 +2273,20 @@
       <c r="L26" s="11" t="inlineStr">
         <is>
           <t>Без изменений — верно + аномалия (пустая карточка)</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>Новую спецификацию в 1С-8 вносит ответственный сотрудник ПО на основании утверждённой «Рабочей инструкции на производство» (форма 16-03).
+Порядок:
+1. Получить утверждённую форму 16-03. Она должна быть утверждена руководителем ЛР / НИМРП / НА либо Техническим директором / Ведущим технологом.
+2. Внести спецификацию в базу 1С-8 в течение одного рабочего дня с момента получения утверждённой формы.
+3. В поле «Статья затрат» выбрать: «Сырье и материалы» — для сырья и товарных компонентов; «Канистры, пробки» — для тары и пакетов; «Этикетки, технологическая информация» — для этикеток.
+4. На вкладке «Дополнительно» установить: «Состояние» — «Утверждён»; «Дата утверждения» — заполняется автоматически; «Ответственный» — заполняется автоматически; «Назначение» — выбрать соответствующее значение: «В состав входит продукция», «Фасовка», «Ароматизаторы НА» либо оставить поле незаполненным, если эти варианты не применяются.
+5. Установить спецификацию как активную.
+6. Во вкладке «Файлы» прикрепить утверждённую форму 16-03: нажать «Добавить»; прикрепить рабочую инструкцию; в поле «Тип документа» выбрать «Документ по продукту».
+7. Нажать «Записать».
+Источник: И-08-05/08 «Внесение спецификаций в базе 1С-8», разделы «Основание для внесения спецификаций», «Порядок внесения спецификаций» и «На вкладке "Дополнительно"».</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clean up dead проход A/B template in tracking xlsx legend sheet
The legend sheet still carried the original план condition table
(Проход A / Проход B) from before the test design changed -- replaced
with the actual test conditions used (model, agent, reasoning, search
scope, collection), matching the same cleanup done in the protocol.
Also removed a leftover stale duplicate row from the first edit pass.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/accounts/eco/pilot-test-03-eco2-tracking.xlsx
+++ b/docs/accounts/eco/pilot-test-03-eco2-tracking.xlsx
@@ -2301,7 +2301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2395,90 +2395,80 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Условия теста — заполнить по факту (см. instrukciya-test-eko-2.md, §6)</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr"/>
+          <t>Условия теста (фактические, 12.09.2026)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Параметр</t>
+          <t>Модель</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Проход A / Проход B</t>
+          <t>OpenAI/gpt-5.5</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Дата и время</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr"/>
+          <t>Агент</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Синапс.Инсайт — Closed-book RAG (системный) — основной; точечные вопросы также задавались агентом «Аналитик (планировщик)» в §1a для сравнения</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Модель</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr"/>
+          <t>Рассуждения (reasoning)</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Выключены</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Агент/режим</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr"/>
+          <t>Область поиска — источники</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Данные (каталог и SQL) + Документы; часть вопросов — только Документы (SQL/каталог выключен), см. протокол</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Рассуждения (reasoning)</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr"/>
+          <t>Область поиска — коллекции</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Основной прогон — только «ЭКО»; точечные перепроверки — переключение на «ЭКО_2» (см. колонку «Коллекция»)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Область поиска — источники</t>
+          <t>Периметр</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>A: Данные (каталог и SQL) + Документы  |  B: только Документы</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Область поиска — коллекции</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Сузить до «ЭКО_2» в обоих проходах</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>Обновлено 12.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>Полный прогон 18/18 вопросов выполнен, коллекция ЭКО (Closed-book RAG системный), с точечными перепроверками на ЭКО_2 для 1.3/2.2/3.2/4.1/5.2/6.2. Подробности — pilot-test-03-eco2-protocol.md.</t>
+          <t>Бейдж «защищённый контур — данные не покидают компании»</t>
         </is>
       </c>
     </row>

</xml_diff>